<commit_message>
generate a downloadable excel file
</commit_message>
<xml_diff>
--- a/backend/downloads/reports/Report_CA2301_2026.xlsx
+++ b/backend/downloads/reports/Report_CA2301_2026.xlsx
@@ -108,10 +108,10 @@
     <t>DIRECTPOATTAINMENT</t>
   </si>
   <si>
-    <t>{"CO1":{"grandTotal":1,"PO1":2,"PO2":2,"PO3":1,"PO4":"","PO5":2,"PO6":"","PO7":1,"PO8":3},"CO2":{"grandTotal":0.5,"PO1":2,"PO2":3,"PO3":2,"PO4":1,"PO5":"","PO6":2,"PO7":"","PO8":1},"CO3":{"grandTotal":0.8,"PO1":1,"PO2":1,"PO3":3,"PO4":2,"PO5":3,"PO6":"","PO7":2,"PO8":""},"CO4":{"grandTotal":1.5,"PO1":3,"PO2":2,"PO3":"","PO4":3,"PO5":1,"PO6":2,"PO7":3,"PO8":2},"CO5":{"grandTotal":2,"PO1":2,"PO2":"","PO3":2,"PO4":1,"PO5":2,"PO6":3,"PO7":1,"PO8":""}}</t>
-  </si>
-  <si>
-    <t>{"PO1":1.23,"PO2":0.91,"PO3":1.05,"PO4":1.23,"PO5":1.24,"PO6":1.43,"PO7":1.3,"PO8":1.08}</t>
+    <t>{"CO1":{"grandTotal":1,"PO1":2,"PO2":2,"PO3":1,"PO4":1,"PO5":2,"PO6":"","PO7":1,"PO8":3},"CO2":{"grandTotal":0.5,"PO1":2,"PO2":3,"PO3":2,"PO4":1,"PO5":"","PO6":2,"PO7":"","PO8":1},"CO3":{"grandTotal":0.8,"PO1":1,"PO2":1,"PO3":3,"PO4":2,"PO5":3,"PO6":"","PO7":2,"PO8":""},"CO4":{"grandTotal":1.5,"PO1":3,"PO2":2,"PO3":"","PO4":3,"PO5":1,"PO6":2,"PO7":3,"PO8":2},"CO5":{"grandTotal":2,"PO1":2,"PO2":"","PO3":2,"PO4":1,"PO5":2,"PO6":3,"PO7":1,"PO8":""}}</t>
+  </si>
+  <si>
+    <t>{"PO1":1.23,"PO2":0.91,"PO3":1.05,"PO4":1.2,"PO5":1.24,"PO6":1.43,"PO7":1.3,"PO8":1.08}</t>
   </si>
 </sst>
 </file>
@@ -1652,7 +1652,7 @@
         <v>27</v>
       </c>
       <c r="B2" s="4">
-        <v>46169.27480583334</v>
+        <v>46179.71537337963</v>
       </c>
       <c r="C2">
         <v>1.16</v>
@@ -1685,7 +1685,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
-        <v>46169.27570399306</v>
+        <v>46179.715983622686</v>
       </c>
       <c r="B2" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
fully prepare download api and resolve the missing value error
</commit_message>
<xml_diff>
--- a/backend/downloads/reports/Report_CA2301_2026.xlsx
+++ b/backend/downloads/reports/Report_CA2301_2026.xlsx
@@ -1924,7 +1924,9 @@
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
-      <c r="I7" s="5"/>
+      <c r="I7" s="5">
+        <v>1.16</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>